<commit_message>
docs: describe the intake agent, its loop breakers, and the counts it moved
Dev_Environment records what shipped and that the agent ships off per branch;
Operations_Findings adds the reply-without-looping rules beside §11's; the
compliance pack carries the four new tables in its counts (re-read from a
fresh database, query beside them) and the agent's replies and per-turn model
reads in the record of processing.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015XGyDiTk9m1NLnqwJVeiVb
</commit_message>
<xml_diff>
--- a/docs/compliance/spreadsheets/CAIQ.xlsx
+++ b/docs/compliance/spreadsheets/CAIQ.xlsx
@@ -1675,7 +1675,7 @@
       </c>
       <c r="E32" s="6" t="inlineStr">
         <is>
-          <t>Enforced by the database: RLS ENABLE and FORCE on 83 of 89 tables, 205 policies, and a database per customer.</t>
+          <t>Enforced by the database: RLS ENABLE and FORCE on 87 of 93 tables, 211 policies, and a database per customer.</t>
         </is>
       </c>
       <c r="F32" s="6" t="inlineStr">
@@ -2315,7 +2315,7 @@
       </c>
       <c r="E52" s="6" t="inlineStr">
         <is>
-          <t>81 audit triggers; vendor support access separately granted, time-boxed, read-only unless the customer grants write scope, logged per transaction.</t>
+          <t>85 audit triggers; vendor support access separately granted, time-boxed, read-only unless the customer grants write scope, logged per transaction.</t>
         </is>
       </c>
       <c r="F52" s="6" t="inlineStr">

</xml_diff>